<commit_message>
Outdoor firmware: divider resistor values as config.h settings, with overdrive checks
P_DIV_TOP_K / P_DIV_BOTTOM_K (default 10k / 20k) and RAIL_DIV_TOP_K / RAIL_DIV_BOTTOM_K
(10k / 15k) set the divider gains, so a board built with 10k everywhere just needs two lines in
config.h. static_asserts refuse values that would push the ADS1115 past its 3.3 V supply (or a
faulted 5 V signal past its 3.6 V maximum), e.g. 22k for R8. The status reports p_div / rail_div.
Parts list notes updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-files/2-parts/HVAC_Monitor_Parts_List.xlsx
+++ b/project-files/2-parts/HVAC_Monitor_Parts_List.xlsx
@@ -2177,7 +2177,11 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="I21" s="49" t="n"/>
+      <c r="I21" s="49" t="inlineStr">
+        <is>
+          <t>R2, R4, R6. 10k also works: set P_DIV_BOTTOM_K 10.0 in config.h</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="27">
       <c r="A22" s="49" t="inlineStr">
@@ -2217,7 +2221,7 @@
       </c>
       <c r="I22" s="49" t="inlineStr">
         <is>
-          <t>Measures 5 V rail for ratiometric correction</t>
+          <t>R7 (10k) / R8 (15k): measures the 5 V rail for ratiometric correction. R8 may be 10k (RAIL_DIV_BOTTOM_K 10.0); 15k is the most it can be</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="30" min="1" max="1"/>
@@ -5255,7 +5259,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="D27" s="51" t="inlineStr">
         <is>
@@ -5267,8 +5270,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" display="Search" r:id="rId1"/>

</xml_diff>

<commit_message>
Parts list: rev B outdoor and indoor board sheets
Adds one sheet per rev B carrier with every board part by reference,
mating plugs, the three SCT-013 CTs and the LoRa antenna, plus a
Summary section for the two boards kept out of the node totals. The
LoRa sheet's module breakout drops to qty 0 now the boards carry the
Wio-SX1262 footprint.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4kWJ9CiBrt94u4WqUxFsk
</commit_message>
<xml_diff>
--- a/project-files/2-parts/HVAC_Monitor_Parts_List.xlsx
+++ b/project-files/2-parts/HVAC_Monitor_Parts_List.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Power Kit" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Outdoor Node" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Indoor Node" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Display Node" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="LoRa Radio" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Infrastructure" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Kit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outdoor Node" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indoor Node" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Display Node" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoRa Radio" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outdoor Board Rev B" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indoor Board Rev B" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -26,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -119,6 +121,10 @@
       <color rgb="FF0563C1"/>
       <sz val="11"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -215,7 +221,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -396,6 +402,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -650,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="30" min="1" max="1"/>
@@ -995,7 +1004,11 @@
       <c r="F18" s="30" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="n"/>
+      <c r="A19" s="61" t="inlineStr">
+        <is>
+          <t>Rev B carrier boards (one board each, parts + plugs + CTs + antenna)</t>
+        </is>
+      </c>
       <c r="B19" s="30" t="n"/>
       <c r="C19" s="30" t="n"/>
       <c r="D19" s="30" t="n"/>
@@ -1003,12 +1016,48 @@
       <c r="F19" s="30" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="n"/>
-      <c r="B20" s="30" t="n"/>
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Outdoor board rev B</t>
+        </is>
+      </c>
+      <c r="B20" s="30">
+        <f>'Outdoor Board Rev B'!$E$50</f>
+        <v/>
+      </c>
       <c r="C20" s="30" t="n"/>
       <c r="D20" s="30" t="n"/>
       <c r="E20" s="30" t="n"/>
       <c r="F20" s="30" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Indoor board rev B</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>'Indoor Board Rev B'!$E$41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Both boards</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>B20+B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>• Not added to the Total above: most of these parts are already counted on the node and LoRa sheets.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1444,6 +1493,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="27">
       <c r="D15" s="42" t="inlineStr">
         <is>
@@ -3211,6 +3261,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51" ht="15" customHeight="1" s="27">
       <c r="D51" s="42" t="inlineStr">
         <is>
@@ -4327,6 +4378,7 @@
       </c>
       <c r="I31" s="49" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="27">
       <c r="D33" s="42" t="inlineStr">
         <is>
@@ -5259,6 +5311,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="D27" s="51" t="inlineStr">
         <is>
@@ -5593,7 +5646,7 @@
         </is>
       </c>
       <c r="C11" s="50" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D11" s="51" t="n">
         <v>3</v>
@@ -5619,7 +5672,7 @@
       </c>
       <c r="I11" s="49" t="inlineStr">
         <is>
-          <t>Until the carrier boards get a LoRa footprint</t>
+          <t>Not needed: rev B boards have the Wio-SX1262 footprint (qty 0 = not in the totals)</t>
         </is>
       </c>
     </row>
@@ -6061,6 +6114,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="D25" s="51" t="inlineStr">
         <is>
@@ -6072,6 +6126,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="57" t="inlineStr">
         <is>
@@ -6520,6 +6575,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="27">
       <c r="D15" s="42" t="inlineStr">
         <is>
@@ -6545,4 +6601,3277 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="27" min="1" max="1"/>
+    <col width="40" customWidth="1" style="27" min="2" max="2"/>
+    <col width="6" customWidth="1" style="27" min="3" max="3"/>
+    <col width="14" customWidth="1" style="27" min="4" max="4"/>
+    <col width="13" customWidth="1" style="27" min="5" max="5"/>
+    <col width="10" customWidth="1" style="27" min="6" max="6"/>
+    <col width="16" customWidth="1" style="27" min="7" max="7"/>
+    <col width="14" customWidth="1" style="27" min="8" max="8"/>
+    <col width="48" customWidth="1" style="27" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="56" t="inlineStr">
+        <is>
+          <t>Outdoor Carrier Rev B — Board Parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="57" t="inlineStr">
+        <is>
+          <t>Blue = editable estimate. Prices are approximate single-unit retail (Oct 2026); links are supplier search pages. Refs match the board silkscreen and fab/*-BOM.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="57" t="inlineStr">
+        <is>
+          <t>Outdoor carrier rev B: 100 x 100 mm. Hand-built with plug-in ESP32, ADS1115 and LM2596 modules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26.85" customHeight="1" s="27">
+      <c r="A4" s="58" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="58" t="inlineStr">
+        <is>
+          <t>Part / Spec</t>
+        </is>
+      </c>
+      <c r="C4" s="58" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="inlineStr">
+        <is>
+          <t>Est. Unit Cost ($)</t>
+        </is>
+      </c>
+      <c r="E4" s="58" t="inlineStr">
+        <is>
+          <t>Line Total ($)</t>
+        </is>
+      </c>
+      <c r="F4" s="58" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="G4" s="58" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="H4" s="58" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I4" s="58" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Controller &amp; power</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n"/>
+      <c r="C5" s="48" t="n"/>
+      <c r="D5" s="48" t="n"/>
+      <c r="E5" s="48" t="n"/>
+      <c r="F5" s="48" t="n"/>
+      <c r="G5" s="48" t="n"/>
+      <c r="H5" s="48" t="n"/>
+      <c r="I5" s="48" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>Bare PCB</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>100 x 100 mm, 2-layer 1.6 mm, JLCPCB (5 pcs per order)</t>
+        </is>
+      </c>
+      <c r="C6" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="52">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G6" s="54" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="H6" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I6" s="49" t="inlineStr">
+        <is>
+          <t>About $15 for 5 boards with shipping; inside JLCPCB's cheapest 100 x 100 mm size. Gerbers: fab/*-JLCPCB-gerbers.zip</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>ESP32 dev board (U1)</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>ESP32-WROOM-32 DevKit, 30-pin, 25.4 mm row spacing</t>
+        </is>
+      </c>
+      <c r="C7" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="52">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G7" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H7" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I7" s="49" t="inlineStr">
+        <is>
+          <t>Check the 25.4 mm (1.0") row spacing before buying</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>Female headers for U1</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>15-pin 2.54 mm female header</t>
+        </is>
+      </c>
+      <c r="C8" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="52">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G8" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H8" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I8" s="49" t="inlineStr">
+        <is>
+          <t>Lets the ESP32 plug in and out</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>Bulk capacitor (C1)</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>470 µF 63 V electrolytic, radial 10 mm, 5 mm pitch</t>
+        </is>
+      </c>
+      <c r="C9" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E9" s="52">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G9" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H9" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I9" s="49" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>TVS diode (D1)</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>SMBJ48CA bidirectional, SMB</t>
+        </is>
+      </c>
+      <c r="C10" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="52">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G10" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I10" s="49" t="inlineStr">
+        <is>
+          <t>Across the 24 VAC input</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>Rectifier diode (D2)</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>1N4007, DO-41</t>
+        </is>
+      </c>
+      <c r="C11" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E11" s="52">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G11" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H11" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I11" s="49" t="inlineStr">
+        <is>
+          <t>Half-wave: keeps C as DC ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>Fuse clips (F1)</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>5x20 mm PCB fuse clip (Littelfuse 111 style)</t>
+        </is>
+      </c>
+      <c r="C12" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="52">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G12" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H12" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I12" s="49" t="inlineStr">
+        <is>
+          <t>Two clips per fuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>Fuse (F1)</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>0.5 A fast-blow, 5x20 mm</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="52">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G13" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H13" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I13" s="49" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>Buck module (U2)</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>LM2596HV module (60 V input), set to 5.00 V before fitting</t>
+        </is>
+      </c>
+      <c r="C14" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="52">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G14" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H14" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I14" s="49" t="inlineStr">
+        <is>
+          <t>Must be the HV version: 24 VAC rectifies to ~40 V peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>Bypass capacitors (C2-C10, C17)</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>0.1 µF ceramic disc, 2.5 mm pitch</t>
+        </is>
+      </c>
+      <c r="C15" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E15" s="52">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G15" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H15" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I15" s="49" t="inlineStr">
+        <is>
+          <t>C17 is the radio decoupling cap listed below; counted here</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>SETUP button (SW1)</t>
+        </is>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>6 mm through-hole tactile switch</t>
+        </is>
+      </c>
+      <c r="C16" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E16" s="52">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G16" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H16" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I16" s="49" t="inlineStr">
+        <is>
+          <t>GPIO14; reserved for Bluetooth setup, no firmware yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="47" t="inlineStr">
+        <is>
+          <t>Sensor inputs</t>
+        </is>
+      </c>
+      <c r="B17" s="48" t="n"/>
+      <c r="C17" s="48" t="n"/>
+      <c r="D17" s="48" t="n"/>
+      <c r="E17" s="48" t="n"/>
+      <c r="F17" s="48" t="n"/>
+      <c r="G17" s="48" t="n"/>
+      <c r="H17" s="48" t="n"/>
+      <c r="I17" s="48" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>ADC module (U3, U4)</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>ADS1115 breakout, 10-pin (0x48 and 0x49)</t>
+        </is>
+      </c>
+      <c r="C18" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="52">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G18" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H18" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I18" s="49" t="inlineStr">
+        <is>
+          <t>Plug-in; 0x48 pressures + rail, 0x49 thermistors</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>Female headers for U3, U4</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>10-pin 2.54 mm female header</t>
+        </is>
+      </c>
+      <c r="C19" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E19" s="52">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G19" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H19" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I19" s="49" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>Divider resistors (R1-R8)</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>10k 1% metal film, ¼ W</t>
+        </is>
+      </c>
+      <c r="C20" s="50" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E20" s="52">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G20" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H20" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I20" s="49" t="inlineStr">
+        <is>
+          <t>Rev B uses 10k for both halves (firmware default)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>Thermistor references (R9, R10, R15, R16)</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>10k 0.1% metal film, ¼ W</t>
+        </is>
+      </c>
+      <c r="C21" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E21" s="52">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G21" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H21" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I21" s="49" t="inlineStr">
+        <is>
+          <t>R15 (true suction) and R16 (discharge) only needed when those thermistors are fitted</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>Mode-input optos (U5, U6)</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>H11AA1, DIP-6</t>
+        </is>
+      </c>
+      <c r="C22" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="51" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E22" s="52">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G22" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H22" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I22" s="49" t="inlineStr">
+        <is>
+          <t>Y and O/B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>DIP-6 sockets for U5, U6</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>6-pin DIP socket, 7.62 mm</t>
+        </is>
+      </c>
+      <c r="C23" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E23" s="52">
+        <f>C23*D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G23" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H23" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I23" s="49" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="49" t="inlineStr">
+        <is>
+          <t>Opto series resistors (R11, R13)</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>4.7k ½ W</t>
+        </is>
+      </c>
+      <c r="C24" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E24" s="52">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G24" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H24" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I24" s="49" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>Opto pull-ups (R12, R14)</t>
+        </is>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>10k ¼ W</t>
+        </is>
+      </c>
+      <c r="C25" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E25" s="52">
+        <f>C25*D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G25" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H25" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I25" s="49" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="47" t="inlineStr">
+        <is>
+          <t>Current sensors (electrical module version 1)</t>
+        </is>
+      </c>
+      <c r="B26" s="48" t="n"/>
+      <c r="C26" s="48" t="n"/>
+      <c r="D26" s="48" t="n"/>
+      <c r="E26" s="48" t="n"/>
+      <c r="F26" s="48" t="n"/>
+      <c r="G26" s="48" t="n"/>
+      <c r="H26" s="48" t="n"/>
+      <c r="I26" s="48" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>CT jacks (J11-J13)</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>CUI SJ1-3523N 3.5 mm stereo jack</t>
+        </is>
+      </c>
+      <c r="C27" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="51" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E27" s="52">
+        <f>C27*D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G27" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H27" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I27" s="49" t="inlineStr">
+        <is>
+          <t>Sits in an edge notch; check fit on a real part</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>CT bias divider (R17, R18)</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>10k + 6.8k 1%, 0805</t>
+        </is>
+      </c>
+      <c r="C28" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E28" s="52">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G28" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H28" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I28" s="49" t="inlineStr">
+        <is>
+          <t>CT_BIAS ≈ 1.34 V</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>CT bias cap (C11)</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>10 µF 16 V electrolytic, radial 5 mm</t>
+        </is>
+      </c>
+      <c r="C29" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E29" s="52">
+        <f>C29*D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G29" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H29" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I29" s="49" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>CT1 burden resistor (R19)</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>18 Ω 1%, 0805</t>
+        </is>
+      </c>
+      <c r="C30" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E30" s="52">
+        <f>C30*D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G30" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H30" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I30" s="49" t="inlineStr">
+        <is>
+          <t>Only CT1 (SCT-013-000) needs a burden; R21, R23 left empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>CT filter resistors (R20, R22, R24)</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>1k, 0805</t>
+        </is>
+      </c>
+      <c r="C31" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E31" s="52">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G31" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H31" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I31" s="49" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>CT filter caps (C12-C14)</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>10 nF, 0805</t>
+        </is>
+      </c>
+      <c r="C32" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E32" s="52">
+        <f>C32*D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G32" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H32" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I32" s="49" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>CT1 compressor</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>SCT-013-000 (100 A, current output)</t>
+        </is>
+      </c>
+      <c r="C33" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="E33" s="52">
+        <f>C33*D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G33" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H33" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I33" s="49" t="inlineStr">
+        <is>
+          <t>Clamps the compressor common</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>CT2 fan</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>SCT-013-005 (5 A / 1 V)</t>
+        </is>
+      </c>
+      <c r="C34" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="E34" s="52">
+        <f>C34*D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G34" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H34" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I34" s="49" t="inlineStr">
+        <is>
+          <t>Condenser fan</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>CT3 HERM</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>SCT-013-010 (10 A / 1 V)</t>
+        </is>
+      </c>
+      <c r="C35" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" s="52">
+        <f>C35*D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G35" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H35" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I35" s="49" t="inlineStr">
+        <is>
+          <t>Run-capacitor HERM lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>Connectors (board side + mating plug)</t>
+        </is>
+      </c>
+      <c r="B36" s="48" t="n"/>
+      <c r="C36" s="48" t="n"/>
+      <c r="D36" s="48" t="n"/>
+      <c r="E36" s="48" t="n"/>
+      <c r="F36" s="48" t="n"/>
+      <c r="G36" s="48" t="n"/>
+      <c r="H36" s="48" t="n"/>
+      <c r="I36" s="48" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>Pluggable terminal (J1)</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/2-G-5.08 header + MC 1,5/2-ST-5.08 plug</t>
+        </is>
+      </c>
+      <c r="C37" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="52">
+        <f>C37*D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G37" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H37" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I37" s="49" t="inlineStr">
+        <is>
+          <t>24 VAC in (R, C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>Pluggable terminal (J2)</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/2-G-5.08 header + MC 1,5/2-ST-5.08 plug</t>
+        </is>
+      </c>
+      <c r="C38" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" s="52">
+        <f>C38*D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G38" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H38" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I38" s="49" t="inlineStr">
+        <is>
+          <t>Y, O/B call inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>Pluggable terminal (J8)</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/4-G-5.08 header + MC 1,5/4-ST-5.08 plug</t>
+        </is>
+      </c>
+      <c r="C39" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="52">
+        <f>C39*D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G39" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H39" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I39" s="49" t="inlineStr">
+        <is>
+          <t>Outdoor air sensor (SHT30 / FS400)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH 3-pin jack (J3-J5)</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>B3B-XH-A vertical + XHP-3 housing + SXH crimps</t>
+        </is>
+      </c>
+      <c r="C40" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E40" s="52">
+        <f>C40*D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G40" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H40" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I40" s="49" t="inlineStr">
+        <is>
+          <t>Pressure transducers: liquid, vapor, true suction (J5 spare until fitted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH 2-pin jack (J6, J7, J9, J10)</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>B2B-XH-A vertical + XHP-2 housing + SXH crimps</t>
+        </is>
+      </c>
+      <c r="C41" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E41" s="52">
+        <f>C41*D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G41" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H41" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I41" s="49" t="inlineStr">
+        <is>
+          <t>Thermistors: suction, liquid, true suction, discharge</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="47" t="inlineStr">
+        <is>
+          <t>LoRa radio and antenna</t>
+        </is>
+      </c>
+      <c r="B42" s="48" t="n"/>
+      <c r="C42" s="48" t="n"/>
+      <c r="D42" s="48" t="n"/>
+      <c r="E42" s="48" t="n"/>
+      <c r="F42" s="48" t="n"/>
+      <c r="G42" s="48" t="n"/>
+      <c r="H42" s="48" t="n"/>
+      <c r="I42" s="48" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="49" t="inlineStr">
+        <is>
+          <t>LoRa module (U7)</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Seeed Wio-SX1262 (FCC Z4T-WIO-SX1262), solders flat on the board</t>
+        </is>
+      </c>
+      <c r="C43" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" s="52">
+        <f>C43*D43</f>
+        <v/>
+      </c>
+      <c r="F43" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G43" s="54" t="inlineStr">
+        <is>
+          <t>Seeed</t>
+        </is>
+      </c>
+      <c r="H43" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I43" s="49" t="inlineStr">
+        <is>
+          <t>Same module as the LoRa Radio sheet; counted there for the node totals</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="49" t="inlineStr">
+        <is>
+          <t>Radio regulator (U8)</t>
+        </is>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>AMS1117-3.3, SOT-223</t>
+        </is>
+      </c>
+      <c r="C44" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E44" s="52">
+        <f>C44*D44</f>
+        <v/>
+      </c>
+      <c r="F44" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G44" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H44" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I44" s="49" t="inlineStr">
+        <is>
+          <t>Own 3.3 V rail for the radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="49" t="inlineStr">
+        <is>
+          <t>Regulator input cap (C15)</t>
+        </is>
+      </c>
+      <c r="B45" s="49" t="inlineStr">
+        <is>
+          <t>10 µF 16 V electrolytic, radial 5 mm</t>
+        </is>
+      </c>
+      <c r="C45" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E45" s="52">
+        <f>C45*D45</f>
+        <v/>
+      </c>
+      <c r="F45" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G45" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H45" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I45" s="49" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="49" t="inlineStr">
+        <is>
+          <t>Regulator output cap (C16)</t>
+        </is>
+      </c>
+      <c r="B46" s="49" t="inlineStr">
+        <is>
+          <t>22 µF 10 V electrolytic, radial 5 mm</t>
+        </is>
+      </c>
+      <c r="C46" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E46" s="52">
+        <f>C46*D46</f>
+        <v/>
+      </c>
+      <c r="F46" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G46" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H46" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I46" s="49" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="49" t="inlineStr">
+        <is>
+          <t>RF pigtail</t>
+        </is>
+      </c>
+      <c r="B47" s="49" t="inlineStr">
+        <is>
+          <t>u.FL (IPEX) to SMA bulkhead, 15 cm</t>
+        </is>
+      </c>
+      <c r="C47" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="52">
+        <f>C47*D47</f>
+        <v/>
+      </c>
+      <c r="F47" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G47" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H47" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I47" s="49" t="inlineStr">
+        <is>
+          <t>Also on the LoRa Radio sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="49" t="inlineStr">
+        <is>
+          <t>915 MHz antenna</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>915 MHz 3 dBi, SMA, outdoor-rated</t>
+        </is>
+      </c>
+      <c r="C48" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="E48" s="52">
+        <f>C48*D48</f>
+        <v/>
+      </c>
+      <c r="F48" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G48" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H48" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I48" s="49" t="inlineStr">
+        <is>
+          <t>Also on the LoRa Radio sheet. Must be 915, not 868</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="D50" s="42" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E50" s="43">
+        <f>SUM(E5:E48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="57" t="inlineStr">
+        <is>
+          <t>• One board each. Sensors, cable and enclosure stay on the Outdoor Node / Indoor Node sheets; the radio and antenna also appear on the LoRa Radio sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="57" t="inlineStr">
+        <is>
+          <t>• So the Summary shows these boards in their own section, outside the node totals, to avoid counting the same parts twice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId39"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="27" min="1" max="1"/>
+    <col width="40" customWidth="1" style="27" min="2" max="2"/>
+    <col width="6" customWidth="1" style="27" min="3" max="3"/>
+    <col width="14" customWidth="1" style="27" min="4" max="4"/>
+    <col width="13" customWidth="1" style="27" min="5" max="5"/>
+    <col width="10" customWidth="1" style="27" min="6" max="6"/>
+    <col width="16" customWidth="1" style="27" min="7" max="7"/>
+    <col width="14" customWidth="1" style="27" min="8" max="8"/>
+    <col width="48" customWidth="1" style="27" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="56" t="inlineStr">
+        <is>
+          <t>Indoor Carrier Rev B — Board Parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="57" t="inlineStr">
+        <is>
+          <t>Blue = editable estimate. Prices are approximate single-unit retail (Oct 2026); links are supplier search pages. Refs match the board silkscreen and fab/*-BOM.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="57" t="inlineStr">
+        <is>
+          <t>Indoor carrier rev B: 100 x 88 mm. Hand-built with plug-in ESP32 and LM2596 modules; TCA9548A soldered on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26.85" customHeight="1" s="27">
+      <c r="A4" s="58" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="58" t="inlineStr">
+        <is>
+          <t>Part / Spec</t>
+        </is>
+      </c>
+      <c r="C4" s="58" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="inlineStr">
+        <is>
+          <t>Est. Unit Cost ($)</t>
+        </is>
+      </c>
+      <c r="E4" s="58" t="inlineStr">
+        <is>
+          <t>Line Total ($)</t>
+        </is>
+      </c>
+      <c r="F4" s="58" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="G4" s="58" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="H4" s="58" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I4" s="58" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Controller &amp; power</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n"/>
+      <c r="C5" s="48" t="n"/>
+      <c r="D5" s="48" t="n"/>
+      <c r="E5" s="48" t="n"/>
+      <c r="F5" s="48" t="n"/>
+      <c r="G5" s="48" t="n"/>
+      <c r="H5" s="48" t="n"/>
+      <c r="I5" s="48" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>Bare PCB</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>100 x 88 mm, 2-layer 1.6 mm, JLCPCB (5 pcs per order)</t>
+        </is>
+      </c>
+      <c r="C6" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="52">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G6" s="54" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="H6" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I6" s="49" t="inlineStr">
+        <is>
+          <t>About $15 for 5 boards with shipping; inside JLCPCB's cheapest 100 x 100 mm size. Gerbers: fab/*-JLCPCB-gerbers.zip</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>ESP32 dev board (U1)</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>ESP32-WROOM-32 DevKit, 30-pin, 25.4 mm row spacing</t>
+        </is>
+      </c>
+      <c r="C7" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="52">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G7" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H7" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I7" s="49" t="inlineStr">
+        <is>
+          <t>Check the 25.4 mm (1.0") row spacing before buying</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>Female headers for U1</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>15-pin 2.54 mm female header</t>
+        </is>
+      </c>
+      <c r="C8" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="52">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G8" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H8" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I8" s="49" t="inlineStr">
+        <is>
+          <t>Lets the ESP32 plug in and out</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>Bulk capacitor (C1)</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>470 µF 63 V electrolytic, radial 10 mm, 5 mm pitch</t>
+        </is>
+      </c>
+      <c r="C9" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E9" s="52">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G9" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H9" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I9" s="49" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>TVS diode (D1)</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>SMBJ48CA bidirectional, SMB</t>
+        </is>
+      </c>
+      <c r="C10" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="52">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G10" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I10" s="49" t="inlineStr">
+        <is>
+          <t>Across the 24 VAC input</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>Rectifier diode (D2)</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>1N4007, DO-41</t>
+        </is>
+      </c>
+      <c r="C11" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E11" s="52">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G11" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H11" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I11" s="49" t="inlineStr">
+        <is>
+          <t>Half-wave: keeps C as DC ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>Fuse clips (F1)</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>5x20 mm PCB fuse clip (Littelfuse 111 style)</t>
+        </is>
+      </c>
+      <c r="C12" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="52">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G12" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H12" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I12" s="49" t="inlineStr">
+        <is>
+          <t>Two clips per fuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>Fuse (F1)</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>0.5 A fast-blow, 5x20 mm</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="52">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G13" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H13" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I13" s="49" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>Buck module (U2)</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>LM2596HV module (60 V input), set to 5.00 V before fitting</t>
+        </is>
+      </c>
+      <c r="C14" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="52">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G14" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H14" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I14" s="49" t="inlineStr">
+        <is>
+          <t>Must be the HV version: 24 VAC rectifies to ~40 V peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>Bypass capacitors (C2, C6)</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>0.1 µF ceramic disc, 2.5 mm pitch</t>
+        </is>
+      </c>
+      <c r="C15" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E15" s="52">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G15" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H15" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I15" s="49" t="inlineStr">
+        <is>
+          <t>C6 is the radio decoupling cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>SETUP button (SW1)</t>
+        </is>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>6 mm through-hole tactile switch</t>
+        </is>
+      </c>
+      <c r="C16" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E16" s="52">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G16" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H16" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I16" s="49" t="inlineStr">
+        <is>
+          <t>GPIO14; reserved for Bluetooth setup, no firmware yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="47" t="inlineStr">
+        <is>
+          <t>Mode inputs and temperature</t>
+        </is>
+      </c>
+      <c r="B17" s="48" t="n"/>
+      <c r="C17" s="48" t="n"/>
+      <c r="D17" s="48" t="n"/>
+      <c r="E17" s="48" t="n"/>
+      <c r="F17" s="48" t="n"/>
+      <c r="G17" s="48" t="n"/>
+      <c r="H17" s="48" t="n"/>
+      <c r="I17" s="48" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Mode-input optos (U3-U6)</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>H11AA1, DIP-6</t>
+        </is>
+      </c>
+      <c r="C18" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E18" s="52">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G18" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H18" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I18" s="49" t="inlineStr">
+        <is>
+          <t>Y, W, G, O/B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>DIP-6 sockets for U3-U6</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>6-pin DIP socket, 7.62 mm</t>
+        </is>
+      </c>
+      <c r="C19" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E19" s="52">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G19" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H19" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I19" s="49" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>Opto series resistors (R2, R4, R6, R8)</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>4.7k ½ W</t>
+        </is>
+      </c>
+      <c r="C20" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E20" s="52">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G20" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H20" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I20" s="49" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>Opto pull-ups (R3, R5, R7, R9)</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>10k ¼ W</t>
+        </is>
+      </c>
+      <c r="C21" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E21" s="52">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G21" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H21" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I21" s="49" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>DS18B20 pull-up (R1)</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>4.7k ¼ W</t>
+        </is>
+      </c>
+      <c r="C22" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E22" s="52">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G22" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H22" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I22" s="49" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="47" t="inlineStr">
+        <is>
+          <t>Sensor hub (humidity + static pressure)</t>
+        </is>
+      </c>
+      <c r="B23" s="48" t="n"/>
+      <c r="C23" s="48" t="n"/>
+      <c r="D23" s="48" t="n"/>
+      <c r="E23" s="48" t="n"/>
+      <c r="F23" s="48" t="n"/>
+      <c r="G23" s="48" t="n"/>
+      <c r="H23" s="48" t="n"/>
+      <c r="I23" s="48" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="49" t="inlineStr">
+        <is>
+          <t>I²C multiplexer (U7)</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>TCA9548A, TSSOP-24 (0x70)</t>
+        </is>
+      </c>
+      <c r="C24" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="51" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E24" s="52">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G24" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H24" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I24" s="49" t="inlineStr">
+        <is>
+          <t>Soldered on the board; replaces the plug-in mux breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>Mux decoupling cap (C3)</t>
+        </is>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>0.1 µF, 0805</t>
+        </is>
+      </c>
+      <c r="C25" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E25" s="52">
+        <f>C25*D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G25" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H25" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I25" s="49" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t>Pull-ups and address (R10-R20)</t>
+        </is>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t>10k, 0805</t>
+        </is>
+      </c>
+      <c r="C26" s="50" t="n">
+        <v>11</v>
+      </c>
+      <c r="D26" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E26" s="52">
+        <f>C26*D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G26" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H26" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I26" s="49" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="47" t="inlineStr">
+        <is>
+          <t>Connectors (board side + mating plug)</t>
+        </is>
+      </c>
+      <c r="B27" s="48" t="n"/>
+      <c r="C27" s="48" t="n"/>
+      <c r="D27" s="48" t="n"/>
+      <c r="E27" s="48" t="n"/>
+      <c r="F27" s="48" t="n"/>
+      <c r="G27" s="48" t="n"/>
+      <c r="H27" s="48" t="n"/>
+      <c r="I27" s="48" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>Pluggable terminal (J1)</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/2-G-5.08 header + MC 1,5/2-ST-5.08 plug</t>
+        </is>
+      </c>
+      <c r="C28" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="52">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G28" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H28" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I28" s="49" t="inlineStr">
+        <is>
+          <t>24 VAC in (R, C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>Pluggable terminal (J2)</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/4-G-5.08 header + MC 1,5/4-ST-5.08 plug</t>
+        </is>
+      </c>
+      <c r="C29" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="52">
+        <f>C29*D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G29" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H29" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I29" s="49" t="inlineStr">
+        <is>
+          <t>Y, W, G, O/B call inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>Pluggable terminal (J5)</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/4-G-5.08 header + MC 1,5/4-ST-5.08 plug</t>
+        </is>
+      </c>
+      <c r="C30" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" s="52">
+        <f>C30*D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G30" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H30" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I30" s="49" t="inlineStr">
+        <is>
+          <t>I²C expansion (spare)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH 3-pin jack (J3, J4)</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>B3B-XH-A vertical + XHP-3 housing + SXH crimps</t>
+        </is>
+      </c>
+      <c r="C31" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E31" s="52">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G31" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H31" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I31" s="49" t="inlineStr">
+        <is>
+          <t>DS18B20 supply and return air</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH 4-pin jack (J6-J10)</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>B4B-XH-A vertical + XHP-4 housing + SXH crimps</t>
+        </is>
+      </c>
+      <c r="C32" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="D32" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E32" s="52">
+        <f>C32*D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G32" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H32" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I32" s="49" t="inlineStr">
+        <is>
+          <t>SHT45 return/supply (ch 0, 1), SDP810 return/supply/filter (ch 2-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>LoRa radio and antenna</t>
+        </is>
+      </c>
+      <c r="B33" s="48" t="n"/>
+      <c r="C33" s="48" t="n"/>
+      <c r="D33" s="48" t="n"/>
+      <c r="E33" s="48" t="n"/>
+      <c r="F33" s="48" t="n"/>
+      <c r="G33" s="48" t="n"/>
+      <c r="H33" s="48" t="n"/>
+      <c r="I33" s="48" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>LoRa module (U8)</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Seeed Wio-SX1262 (FCC Z4T-WIO-SX1262), solders flat on the board</t>
+        </is>
+      </c>
+      <c r="C34" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E34" s="52">
+        <f>C34*D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G34" s="54" t="inlineStr">
+        <is>
+          <t>Seeed</t>
+        </is>
+      </c>
+      <c r="H34" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I34" s="49" t="inlineStr">
+        <is>
+          <t>Same module as the LoRa Radio sheet; counted there for the node totals</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>Radio regulator (U9)</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>AMS1117-3.3, SOT-223</t>
+        </is>
+      </c>
+      <c r="C35" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E35" s="52">
+        <f>C35*D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G35" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H35" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I35" s="49" t="inlineStr">
+        <is>
+          <t>Own 3.3 V rail for the radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>Regulator input cap (C4)</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>10 µF 16 V electrolytic, radial 5 mm</t>
+        </is>
+      </c>
+      <c r="C36" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E36" s="52">
+        <f>C36*D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G36" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H36" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I36" s="49" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>Regulator output cap (C5)</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>22 µF 10 V electrolytic, radial 5 mm</t>
+        </is>
+      </c>
+      <c r="C37" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E37" s="52">
+        <f>C37*D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G37" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H37" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I37" s="49" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>RF pigtail</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>u.FL (IPEX) to SMA bulkhead, 15 cm</t>
+        </is>
+      </c>
+      <c r="C38" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" s="52">
+        <f>C38*D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G38" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H38" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I38" s="49" t="inlineStr">
+        <is>
+          <t>Also on the LoRa Radio sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>915 MHz antenna</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>915 MHz 3 dBi, SMA, outdoor-rated</t>
+        </is>
+      </c>
+      <c r="C39" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="E39" s="52">
+        <f>C39*D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="59" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G39" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H39" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I39" s="49" t="inlineStr">
+        <is>
+          <t>Also on the LoRa Radio sheet. Must be 915, not 868</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="D41" s="42" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E41" s="43">
+        <f>SUM(E5:E39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="57" t="inlineStr">
+        <is>
+          <t>• One board each. Sensors, cable and enclosure stay on the Outdoor Node / Indoor Node sheets; the radio and antenna also appear on the LoRa Radio sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="57" t="inlineStr">
+        <is>
+          <t>• So the Summary shows these boards in their own section, outside the node totals, to avoid counting the same parts twice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId30"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Parts list: rev B carrier board sheets (outdoor, indoor) and a rev B block on the summary
Outdoor Carrier Rev B and Indoor Carrier Rev B list every part on each rev B board
(from the fab BOMs, refs as on the silkscreen) plus the mating plugs, housings, sockets,
the bare PCB and the SCT-013 clamps, in the node sheets' format (blue estimates, phase,
supplier search links). The summary totals them separately, since they overlap the node
sheets. Existing sheets are unchanged.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4kWJ9CiBrt94u4WqUxFsk
</commit_message>
<xml_diff>
--- a/project-files/2-parts/HVAC_Monitor_Parts_List.xlsx
+++ b/project-files/2-parts/HVAC_Monitor_Parts_List.xlsx
@@ -11,9 +11,11 @@
     <sheet name="Power Kit" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Outdoor Node" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Indoor Node" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Display Node" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="LoRa Radio" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Infrastructure" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Outdoor Carrier Rev B" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Indoor Carrier Rev B" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Display Node" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="LoRa Radio" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Infrastructure" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -26,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -119,6 +121,11 @@
       <color rgb="FF0563C1"/>
       <sz val="11"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="11">
@@ -215,7 +222,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -396,6 +403,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -650,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="30" min="1" max="1"/>
@@ -995,7 +1005,11 @@
       <c r="F18" s="30" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="n"/>
+      <c r="A19" s="61" t="inlineStr">
+        <is>
+          <t>Rev B carrier boards (per-board build: bare PCB + everything soldered or plugged onto it)</t>
+        </is>
+      </c>
       <c r="B19" s="30" t="n"/>
       <c r="C19" s="30" t="n"/>
       <c r="D19" s="30" t="n"/>
@@ -1003,12 +1017,155 @@
       <c r="F19" s="30" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="n"/>
-      <c r="B20" s="30" t="n"/>
-      <c r="C20" s="30" t="n"/>
-      <c r="D20" s="30" t="n"/>
-      <c r="E20" s="30" t="n"/>
-      <c r="F20" s="30" t="n"/>
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Node</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>V1 (core)</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="F20" s="30" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>All Items</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Outdoor Carrier Rev B</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>SUMIFS('Outdoor Carrier Rev B'!$E$5:$E$51,'Outdoor Carrier Rev B'!$F$5:$F$51,"V1")</f>
+        <v/>
+      </c>
+      <c r="C21">
+        <f>SUMIFS('Outdoor Carrier Rev B'!$E$5:$E$51,'Outdoor Carrier Rev B'!$F$5:$F$51,"Optional")</f>
+        <v/>
+      </c>
+      <c r="D21">
+        <f>SUMIFS('Outdoor Carrier Rev B'!$E$5:$E$51,'Outdoor Carrier Rev B'!$F$5:$F$51,"Phase 2")</f>
+        <v/>
+      </c>
+      <c r="E21">
+        <f>SUMIFS('Outdoor Carrier Rev B'!$E$5:$E$51,'Outdoor Carrier Rev B'!$F$5:$F$51,"Future")</f>
+        <v/>
+      </c>
+      <c r="F21">
+        <f>SUMIFS('Outdoor Carrier Rev B'!$E$5:$E$51,'Outdoor Carrier Rev B'!$F$5:$F$51,"LoRa")</f>
+        <v/>
+      </c>
+      <c r="G21">
+        <f>SUM(B21:F21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Indoor Carrier Rev B</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>SUMIFS('Indoor Carrier Rev B'!$E$5:$E$41,'Indoor Carrier Rev B'!$F$5:$F$41,"V1")</f>
+        <v/>
+      </c>
+      <c r="C22">
+        <f>SUMIFS('Indoor Carrier Rev B'!$E$5:$E$41,'Indoor Carrier Rev B'!$F$5:$F$41,"Optional")</f>
+        <v/>
+      </c>
+      <c r="D22">
+        <f>SUMIFS('Indoor Carrier Rev B'!$E$5:$E$41,'Indoor Carrier Rev B'!$F$5:$F$41,"Phase 2")</f>
+        <v/>
+      </c>
+      <c r="E22">
+        <f>SUMIFS('Indoor Carrier Rev B'!$E$5:$E$41,'Indoor Carrier Rev B'!$F$5:$F$41,"Future")</f>
+        <v/>
+      </c>
+      <c r="F22">
+        <f>SUMIFS('Indoor Carrier Rev B'!$E$5:$E$41,'Indoor Carrier Rev B'!$F$5:$F$41,"LoRa")</f>
+        <v/>
+      </c>
+      <c r="G22">
+        <f>SUM(B22:F22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Rev B boards total</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>SUM(B21:B22)</f>
+        <v/>
+      </c>
+      <c r="C23">
+        <f>SUM(C21:C22)</f>
+        <v/>
+      </c>
+      <c r="D23">
+        <f>SUM(D21:D22)</f>
+        <v/>
+      </c>
+      <c r="E23">
+        <f>SUM(E21:E22)</f>
+        <v/>
+      </c>
+      <c r="F23">
+        <f>SUM(F21:F22)</f>
+        <v/>
+      </c>
+      <c r="G23">
+        <f>SUM(G21:G22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>• The rev B sheets overlap the node sheets (ESP32, power kit parts, ADS1115, optos, resistors, TCA9548A): they are a shopping list for building one board, so they are not added to the totals above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>• Rev B puts the TCA9548A, the LoRa module footprint and three CT jacks on the boards: the LoRa sheet's "Module breakout" and the Indoor Node sheet's TCA9548A breakout are not needed with rev B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>• The CT clamps (SCT-013-000 / -005 / -010) are electrical module version 1 and sit in the Phase 2 column.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -4371,6 +4528,3454 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="27" min="1" max="1"/>
+    <col width="40" customWidth="1" style="27" min="2" max="2"/>
+    <col width="6" customWidth="1" style="27" min="3" max="3"/>
+    <col width="14" customWidth="1" style="27" min="4" max="4"/>
+    <col width="13" customWidth="1" style="27" min="5" max="5"/>
+    <col width="10" customWidth="1" style="27" min="6" max="6"/>
+    <col width="16" customWidth="1" style="27" min="7" max="7"/>
+    <col width="14" customWidth="1" style="27" min="8" max="8"/>
+    <col width="48" customWidth="1" style="27" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="56" t="inlineStr">
+        <is>
+          <t>Outdoor Carrier Rev B — Board Parts List</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="57" t="inlineStr">
+        <is>
+          <t>Blue = editable estimate. Prices are approximate single-unit retail (Oct 2026); links are supplier search pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="57" t="inlineStr">
+        <is>
+          <t>Everything on the rev B outdoor board, from hardware/outdoor-carrier/fab/outdoor-carrier-BOM.csv (branch claude/rev-b). Refs match the silkscreen. Sensors that plug in are on the Outdoor Node sheet, except the CT clamps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26.85" customHeight="1" s="27">
+      <c r="A4" s="58" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="58" t="inlineStr">
+        <is>
+          <t>Part / Spec</t>
+        </is>
+      </c>
+      <c r="C4" s="58" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="inlineStr">
+        <is>
+          <t>Est. Unit Cost ($)</t>
+        </is>
+      </c>
+      <c r="E4" s="58" t="inlineStr">
+        <is>
+          <t>Line Total ($)</t>
+        </is>
+      </c>
+      <c r="F4" s="58" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="G4" s="58" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="H4" s="58" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I4" s="58" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Board</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n"/>
+      <c r="C5" s="48" t="n"/>
+      <c r="D5" s="48" t="n"/>
+      <c r="E5" s="48" t="n"/>
+      <c r="F5" s="48" t="n"/>
+      <c r="G5" s="48" t="n"/>
+      <c r="H5" s="48" t="n"/>
+      <c r="I5" s="48" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>Bare PCB</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>Outdoor carrier rev B, 100 × 100 mm, 2-layer 1.6 mm</t>
+        </is>
+      </c>
+      <c r="C6" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="52">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G6" s="54" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="H6" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I6" s="49" t="inlineStr">
+        <is>
+          <t>Upload fab/outdoor-carrier-JLCPCB-gerbers.zip. About $2 for 5 boards at this size, plus shipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="47" t="inlineStr">
+        <is>
+          <t>Plug-in modules and sockets</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="n"/>
+      <c r="C7" s="48" t="n"/>
+      <c r="D7" s="48" t="n"/>
+      <c r="E7" s="48" t="n"/>
+      <c r="F7" s="48" t="n"/>
+      <c r="G7" s="48" t="n"/>
+      <c r="H7" s="48" t="n"/>
+      <c r="I7" s="48" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>ESP32 dev board</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>ESP32 DevKit 30-pin, ESP-WROOM-32 (U1)</t>
+        </is>
+      </c>
+      <c r="C8" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="52">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G8" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H8" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I8" s="49" t="inlineStr">
+        <is>
+          <t>Same board as rev A; antenna end overhangs the left edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>Buck converter module</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>LM2596HV (60 V input) (U2)</t>
+        </is>
+      </c>
+      <c r="C9" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="52">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G9" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H9" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I9" s="49" t="inlineStr">
+        <is>
+          <t>Set to 5.00 V before plugging in</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>ADC module</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>ADS1115 16-bit, 4-ch (U3 0x48, U4 0x49)</t>
+        </is>
+      </c>
+      <c r="C10" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="52">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G10" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I10" s="49" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>LoRa radio module</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>Seeed Wio-SX1262 with u.FL (U7)</t>
+        </is>
+      </c>
+      <c r="C11" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" s="52">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="39" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G11" s="54" t="inlineStr">
+        <is>
+          <t>Seeed</t>
+        </is>
+      </c>
+      <c r="H11" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I11" s="49" t="inlineStr">
+        <is>
+          <t>Solders onto the board (castellated pads). Antenna + pigtail are on the LoRa Radio sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>AC-input optocoupler</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>H11AA1 (U5, U6)</t>
+        </is>
+      </c>
+      <c r="C12" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="51" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E12" s="52">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G12" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H12" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I12" s="49" t="inlineStr">
+        <is>
+          <t>Y and O/B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>Female header 1×15</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>2.54 mm pitch</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E13" s="52">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G13" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H13" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I13" s="49" t="inlineStr">
+        <is>
+          <t>ESP32 sockets</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>Female header 1×10</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>2.54 mm pitch</t>
+        </is>
+      </c>
+      <c r="C14" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="52">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G14" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H14" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I14" s="49" t="inlineStr">
+        <is>
+          <t>ADS1115 sockets</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>Single-pin socket</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>2.54 mm female header, 1 pin (or cut from a strip)</t>
+        </is>
+      </c>
+      <c r="C15" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E15" s="52">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G15" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H15" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I15" s="49" t="inlineStr">
+        <is>
+          <t>LM2596 module corners</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>DIP-6 socket</t>
+        </is>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>7.62 mm</t>
+        </is>
+      </c>
+      <c r="C16" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E16" s="52">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G16" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H16" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I16" s="49" t="inlineStr">
+        <is>
+          <t>Optos</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="47" t="inlineStr">
+        <is>
+          <t>24 VAC supply and radio regulator</t>
+        </is>
+      </c>
+      <c r="B17" s="48" t="n"/>
+      <c r="C17" s="48" t="n"/>
+      <c r="D17" s="48" t="n"/>
+      <c r="E17" s="48" t="n"/>
+      <c r="F17" s="48" t="n"/>
+      <c r="G17" s="48" t="n"/>
+      <c r="H17" s="48" t="n"/>
+      <c r="I17" s="48" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Fuse clips</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>Littelfuse 111 series, 5×20 mm PCB clip (F1)</t>
+        </is>
+      </c>
+      <c r="C18" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E18" s="52">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G18" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H18" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I18" s="49" t="inlineStr">
+        <is>
+          <t>Two per fuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>Fuse</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>0.5 A fast-blow, 5×20 mm</t>
+        </is>
+      </c>
+      <c r="C19" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E19" s="52">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G19" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H19" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I19" s="49" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>TVS diode</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>SMBJ48CA bidirectional (D1)</t>
+        </is>
+      </c>
+      <c r="C20" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E20" s="52">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G20" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H20" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I20" s="49" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>Rectifier diode</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>1N4007 (D2)</t>
+        </is>
+      </c>
+      <c r="C21" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E21" s="52">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G21" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H21" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I21" s="49" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>Bulk capacitor</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>470 µF 63 V electrolytic, 10 mm, 5 mm pitch (C1)</t>
+        </is>
+      </c>
+      <c r="C22" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E22" s="52">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G22" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H22" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I22" s="49" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>Radio regulator</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>AMS1117-3.3, SOT-223 (U8)</t>
+        </is>
+      </c>
+      <c r="C23" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E23" s="52">
+        <f>C23*D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="39" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G23" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H23" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I23" s="49" t="inlineStr">
+        <is>
+          <t>Radio-only 3.3 V rail</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="49" t="inlineStr">
+        <is>
+          <t>Electrolytic capacitor</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>10 µF 16 V, 5 mm, 2 mm pitch (C11, C15)</t>
+        </is>
+      </c>
+      <c r="C24" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E24" s="52">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G24" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H24" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I24" s="49" t="inlineStr">
+        <is>
+          <t>C11 CT bias, C15 regulator input</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>Electrolytic capacitor</t>
+        </is>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>22 µF 10 V, 5 mm, 2 mm pitch (C16)</t>
+        </is>
+      </c>
+      <c r="C25" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E25" s="52">
+        <f>C25*D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="39" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G25" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H25" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I25" s="49" t="inlineStr">
+        <is>
+          <t>Regulator output</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t>SETUP button</t>
+        </is>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t>6 × 6 mm tact switch, 5 mm tall, THT (SW1)</t>
+        </is>
+      </c>
+      <c r="C26" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E26" s="52">
+        <f>C26*D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G26" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H26" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I26" s="49" t="inlineStr">
+        <is>
+          <t>Pressed through the lid by the printed plunger</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="47" t="inlineStr">
+        <is>
+          <t>Through-hole passives</t>
+        </is>
+      </c>
+      <c r="B27" s="48" t="n"/>
+      <c r="C27" s="48" t="n"/>
+      <c r="D27" s="48" t="n"/>
+      <c r="E27" s="48" t="n"/>
+      <c r="F27" s="48" t="n"/>
+      <c r="G27" s="48" t="n"/>
+      <c r="H27" s="48" t="n"/>
+      <c r="I27" s="48" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>Disc capacitor</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>0.1 µF 50 V ceramic, 2.5 mm pitch (C2–C10, C17)</t>
+        </is>
+      </c>
+      <c r="C28" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="D28" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E28" s="52">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G28" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H28" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I28" s="49" t="inlineStr">
+        <is>
+          <t>Bypass and ADC input filters</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>Divider resistor</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>10k 1% ¼ W metal film (R1–R8)</t>
+        </is>
+      </c>
+      <c r="C29" s="50" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E29" s="52">
+        <f>C29*D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G29" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H29" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I29" s="49" t="inlineStr">
+        <is>
+          <t>Three pressure dividers + 5 V rail monitor, all 10k</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>Thermistor reference resistor</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>10k 0.1% ¼ W (R9, R10, R15, R16)</t>
+        </is>
+      </c>
+      <c r="C30" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E30" s="52">
+        <f>C30*D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G30" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H30" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I30" s="49" t="inlineStr">
+        <is>
+          <t>One per thermistor input, incl. discharge</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>Opto series resistor</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>4.7k ½ W (R11, R13)</t>
+        </is>
+      </c>
+      <c r="C31" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E31" s="52">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G31" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H31" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I31" s="49" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>Opto pull-up resistor</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>10k ¼ W (R12, R14)</t>
+        </is>
+      </c>
+      <c r="C32" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E32" s="52">
+        <f>C32*D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G32" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H32" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I32" s="49" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>CT inputs (electrical module version 1)</t>
+        </is>
+      </c>
+      <c r="B33" s="48" t="n"/>
+      <c r="C33" s="48" t="n"/>
+      <c r="D33" s="48" t="n"/>
+      <c r="E33" s="48" t="n"/>
+      <c r="F33" s="48" t="n"/>
+      <c r="G33" s="48" t="n"/>
+      <c r="H33" s="48" t="n"/>
+      <c r="I33" s="48" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>3.5 mm jack</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>CUI SJ1-3523N, horizontal (J11–J13)</t>
+        </is>
+      </c>
+      <c r="C34" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="52">
+        <f>C34*D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G34" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H34" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I34" s="49" t="inlineStr">
+        <is>
+          <t>Left board edge; plugs go through the box wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>Bias resistor</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>10k 1% 0805 (R17)</t>
+        </is>
+      </c>
+      <c r="C35" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E35" s="52">
+        <f>C35*D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G35" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H35" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I35" s="49" t="inlineStr">
+        <is>
+          <t>CT_BIAS 1.34 V</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>Bias resistor</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>6.8k 1% 0805 (R18)</t>
+        </is>
+      </c>
+      <c r="C36" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E36" s="52">
+        <f>C36*D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G36" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H36" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I36" s="49" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>Burden resistor</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>18 Ω 1% 0805 (R19)</t>
+        </is>
+      </c>
+      <c r="C37" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E37" s="52">
+        <f>C37*D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G37" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H37" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I37" s="49" t="inlineStr">
+        <is>
+          <t>CT1 only. R21/R23 stay empty for the voltage-output clamps</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>Series resistor</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>1k 0805 (R20, R22, R24)</t>
+        </is>
+      </c>
+      <c r="C38" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E38" s="52">
+        <f>C38*D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G38" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H38" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I38" s="49" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>Filter capacitor</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>10 nF 0805 (C12–C14)</t>
+        </is>
+      </c>
+      <c r="C39" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E39" s="52">
+        <f>C39*D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G39" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H39" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I39" s="49" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>CT clamp, compressor</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>SCT-013-000, 100 A : 50 mA</t>
+        </is>
+      </c>
+      <c r="C40" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E40" s="52">
+        <f>C40*D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G40" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H40" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I40" s="49" t="inlineStr">
+        <is>
+          <t>Plugs into J11 (CT1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>CT clamp, condenser fan</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>SCT-013-005, 5 A : 1 V</t>
+        </is>
+      </c>
+      <c r="C41" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E41" s="52">
+        <f>C41*D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G41" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H41" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I41" s="49" t="inlineStr">
+        <is>
+          <t>Plugs into J12 (CT2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>CT clamp, HERM lead</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>SCT-013-010, 10 A : 1 V</t>
+        </is>
+      </c>
+      <c r="C42" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E42" s="52">
+        <f>C42*D42</f>
+        <v/>
+      </c>
+      <c r="F42" s="39" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G42" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H42" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I42" s="49" t="inlineStr">
+        <is>
+          <t>Plugs into J13 (CT3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="47" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="B43" s="48" t="n"/>
+      <c r="C43" s="48" t="n"/>
+      <c r="D43" s="48" t="n"/>
+      <c r="E43" s="48" t="n"/>
+      <c r="F43" s="48" t="n"/>
+      <c r="G43" s="48" t="n"/>
+      <c r="H43" s="48" t="n"/>
+      <c r="I43" s="48" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="49" t="inlineStr">
+        <is>
+          <t>Terminal header, 2-pos</t>
+        </is>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/2-G-5,08 (J1, J2)</t>
+        </is>
+      </c>
+      <c r="C44" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" s="51" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E44" s="52">
+        <f>C44*D44</f>
+        <v/>
+      </c>
+      <c r="F44" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G44" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H44" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I44" s="49" t="inlineStr">
+        <is>
+          <t>24 VAC in; Y and O/B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="49" t="inlineStr">
+        <is>
+          <t>Terminal plug, 2-pos</t>
+        </is>
+      </c>
+      <c r="B45" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/2-ST-5,08</t>
+        </is>
+      </c>
+      <c r="C45" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="51" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E45" s="52">
+        <f>C45*D45</f>
+        <v/>
+      </c>
+      <c r="F45" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G45" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H45" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I45" s="49" t="inlineStr">
+        <is>
+          <t>Mates J1, J2</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="49" t="inlineStr">
+        <is>
+          <t>Terminal header, 4-pos</t>
+        </is>
+      </c>
+      <c r="B46" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/4-G-5,08 (J8)</t>
+        </is>
+      </c>
+      <c r="C46" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" s="52">
+        <f>C46*D46</f>
+        <v/>
+      </c>
+      <c r="F46" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G46" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H46" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I46" s="49" t="inlineStr">
+        <is>
+          <t>SHT30 probe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="49" t="inlineStr">
+        <is>
+          <t>Terminal plug, 4-pos</t>
+        </is>
+      </c>
+      <c r="B47" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/4-ST-5,08</t>
+        </is>
+      </c>
+      <c r="C47" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="51" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E47" s="52">
+        <f>C47*D47</f>
+        <v/>
+      </c>
+      <c r="F47" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G47" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H47" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I47" s="49" t="inlineStr">
+        <is>
+          <t>Mates J8</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH header, 3-pin</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>B3B-XH-A (J3–J5)</t>
+        </is>
+      </c>
+      <c r="C48" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E48" s="52">
+        <f>C48*D48</f>
+        <v/>
+      </c>
+      <c r="F48" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G48" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H48" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I48" s="49" t="inlineStr">
+        <is>
+          <t>Pressure transducers</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH header, 2-pin</t>
+        </is>
+      </c>
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>B2B-XH-A (J6, J7, J9, J10)</t>
+        </is>
+      </c>
+      <c r="C49" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" s="51" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E49" s="52">
+        <f>C49*D49</f>
+        <v/>
+      </c>
+      <c r="F49" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G49" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H49" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I49" s="49" t="inlineStr">
+        <is>
+          <t>Thermistors</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH housing, 3-pin</t>
+        </is>
+      </c>
+      <c r="B50" s="49" t="inlineStr">
+        <is>
+          <t>XHP-3 + SXH-001T-P0.6 crimps</t>
+        </is>
+      </c>
+      <c r="C50" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E50" s="52">
+        <f>C50*D50</f>
+        <v/>
+      </c>
+      <c r="F50" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G50" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H50" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I50" s="49" t="inlineStr">
+        <is>
+          <t>Cable side</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH housing, 2-pin</t>
+        </is>
+      </c>
+      <c r="B51" s="49" t="inlineStr">
+        <is>
+          <t>XHP-2 + SXH-001T-P0.6 crimps</t>
+        </is>
+      </c>
+      <c r="C51" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E51" s="52">
+        <f>C51*D51</f>
+        <v/>
+      </c>
+      <c r="F51" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G51" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H51" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I51" s="49" t="inlineStr">
+        <is>
+          <t>Cable side</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="D53" s="42" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E53" s="43">
+        <f>SUM(E5:E51)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId41"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="27" min="1" max="1"/>
+    <col width="40" customWidth="1" style="27" min="2" max="2"/>
+    <col width="6" customWidth="1" style="27" min="3" max="3"/>
+    <col width="14" customWidth="1" style="27" min="4" max="4"/>
+    <col width="13" customWidth="1" style="27" min="5" max="5"/>
+    <col width="10" customWidth="1" style="27" min="6" max="6"/>
+    <col width="16" customWidth="1" style="27" min="7" max="7"/>
+    <col width="14" customWidth="1" style="27" min="8" max="8"/>
+    <col width="48" customWidth="1" style="27" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="56" t="inlineStr">
+        <is>
+          <t>Indoor Carrier Rev B — Board Parts List</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="57" t="inlineStr">
+        <is>
+          <t>Blue = editable estimate. Prices are approximate single-unit retail (Oct 2026); links are supplier search pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="57" t="inlineStr">
+        <is>
+          <t>Everything on the rev B indoor board, from hardware/indoor-carrier/fab/indoor-carrier-BOM.csv (branch claude/rev-b). Refs match the silkscreen. Probes and sensors that plug in are on the Indoor Node sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26.85" customHeight="1" s="27">
+      <c r="A4" s="58" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="58" t="inlineStr">
+        <is>
+          <t>Part / Spec</t>
+        </is>
+      </c>
+      <c r="C4" s="58" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="inlineStr">
+        <is>
+          <t>Est. Unit Cost ($)</t>
+        </is>
+      </c>
+      <c r="E4" s="58" t="inlineStr">
+        <is>
+          <t>Line Total ($)</t>
+        </is>
+      </c>
+      <c r="F4" s="58" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="G4" s="58" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="H4" s="58" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I4" s="58" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Board</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n"/>
+      <c r="C5" s="48" t="n"/>
+      <c r="D5" s="48" t="n"/>
+      <c r="E5" s="48" t="n"/>
+      <c r="F5" s="48" t="n"/>
+      <c r="G5" s="48" t="n"/>
+      <c r="H5" s="48" t="n"/>
+      <c r="I5" s="48" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>Bare PCB</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>Indoor carrier rev B, 100 × 88 mm, 2-layer 1.6 mm</t>
+        </is>
+      </c>
+      <c r="C6" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="52">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G6" s="54" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="H6" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I6" s="49" t="inlineStr">
+        <is>
+          <t>Upload fab/indoor-carrier-JLCPCB-gerbers.zip. About $2 for 5 boards at this size, plus shipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="47" t="inlineStr">
+        <is>
+          <t>Plug-in modules, chips and sockets</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="n"/>
+      <c r="C7" s="48" t="n"/>
+      <c r="D7" s="48" t="n"/>
+      <c r="E7" s="48" t="n"/>
+      <c r="F7" s="48" t="n"/>
+      <c r="G7" s="48" t="n"/>
+      <c r="H7" s="48" t="n"/>
+      <c r="I7" s="48" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>ESP32 dev board</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>ESP32 DevKit 30-pin, ESP-WROOM-32 (U1)</t>
+        </is>
+      </c>
+      <c r="C8" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="52">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G8" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H8" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I8" s="49" t="inlineStr">
+        <is>
+          <t>Same board as rev A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>Buck converter module</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>LM2596HV (60 V input) (U2)</t>
+        </is>
+      </c>
+      <c r="C9" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="52">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G9" s="54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="H9" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I9" s="49" t="inlineStr">
+        <is>
+          <t>Set to 5.00 V before plugging in</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>LoRa radio module</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>Seeed Wio-SX1262 with u.FL (U8)</t>
+        </is>
+      </c>
+      <c r="C10" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" s="52">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="39" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G10" s="54" t="inlineStr">
+        <is>
+          <t>Seeed</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I10" s="49" t="inlineStr">
+        <is>
+          <t>Solders onto the board (castellated pads). Antenna + pigtail are on the LoRa Radio sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>I²C multiplexer chip</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>TCA9548APWR, TSSOP-24 (U7)</t>
+        </is>
+      </c>
+      <c r="C11" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="51" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="52">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G11" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H11" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I11" s="49" t="inlineStr">
+        <is>
+          <t>On the board now (address 0x70); replaces the TCA9548A breakout on the Indoor Node sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>AC-input optocoupler</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>H11AA1 (U3–U6)</t>
+        </is>
+      </c>
+      <c r="C12" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="51" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E12" s="52">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G12" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H12" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I12" s="49" t="inlineStr">
+        <is>
+          <t>Y, W, G, O/B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>Female header 1×15</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>2.54 mm pitch</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E13" s="52">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G13" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H13" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I13" s="49" t="inlineStr">
+        <is>
+          <t>ESP32 sockets</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>Single-pin socket</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>2.54 mm female header, 1 pin (or cut from a strip)</t>
+        </is>
+      </c>
+      <c r="C14" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E14" s="52">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G14" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H14" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I14" s="49" t="inlineStr">
+        <is>
+          <t>LM2596 module corners</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>DIP-6 socket</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>7.62 mm</t>
+        </is>
+      </c>
+      <c r="C15" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E15" s="52">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G15" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H15" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I15" s="49" t="inlineStr">
+        <is>
+          <t>Optos</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="47" t="inlineStr">
+        <is>
+          <t>24 VAC supply and radio regulator</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="n"/>
+      <c r="C16" s="48" t="n"/>
+      <c r="D16" s="48" t="n"/>
+      <c r="E16" s="48" t="n"/>
+      <c r="F16" s="48" t="n"/>
+      <c r="G16" s="48" t="n"/>
+      <c r="H16" s="48" t="n"/>
+      <c r="I16" s="48" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>Fuse clips</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Littelfuse 111 series, 5×20 mm PCB clip (F1)</t>
+        </is>
+      </c>
+      <c r="C17" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E17" s="52">
+        <f>C17*D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G17" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H17" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I17" s="49" t="inlineStr">
+        <is>
+          <t>Two per fuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Fuse</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>0.5 A fast-blow, 5×20 mm</t>
+        </is>
+      </c>
+      <c r="C18" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E18" s="52">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G18" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H18" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I18" s="49" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>TVS diode</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>SMBJ48CA bidirectional (D1)</t>
+        </is>
+      </c>
+      <c r="C19" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E19" s="52">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G19" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H19" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I19" s="49" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>Rectifier diode</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>1N4007 (D2)</t>
+        </is>
+      </c>
+      <c r="C20" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E20" s="52">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G20" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H20" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I20" s="49" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>Bulk capacitor</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>470 µF 63 V electrolytic, 10 mm, 5 mm pitch (C1)</t>
+        </is>
+      </c>
+      <c r="C21" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E21" s="52">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G21" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H21" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I21" s="49" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>Radio regulator</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>AMS1117-3.3, SOT-223 (U9)</t>
+        </is>
+      </c>
+      <c r="C22" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E22" s="52">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="39" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G22" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H22" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I22" s="49" t="inlineStr">
+        <is>
+          <t>Radio-only 3.3 V rail</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>Electrolytic capacitor</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>10 µF 16 V, 5 mm, 2 mm pitch (C4)</t>
+        </is>
+      </c>
+      <c r="C23" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E23" s="52">
+        <f>C23*D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="39" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G23" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H23" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I23" s="49" t="inlineStr">
+        <is>
+          <t>Regulator input</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="49" t="inlineStr">
+        <is>
+          <t>Electrolytic capacitor</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>22 µF 10 V, 5 mm, 2 mm pitch (C5)</t>
+        </is>
+      </c>
+      <c r="C24" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E24" s="52">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="39" t="inlineStr">
+        <is>
+          <t>LoRa</t>
+        </is>
+      </c>
+      <c r="G24" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H24" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I24" s="49" t="inlineStr">
+        <is>
+          <t>Regulator output</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>SETUP button</t>
+        </is>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>6 × 6 mm tact switch, 5 mm tall, THT (SW1)</t>
+        </is>
+      </c>
+      <c r="C25" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E25" s="52">
+        <f>C25*D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G25" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H25" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I25" s="49" t="inlineStr">
+        <is>
+          <t>Pressed through the lid by the printed plunger</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="47" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="B26" s="48" t="n"/>
+      <c r="C26" s="48" t="n"/>
+      <c r="D26" s="48" t="n"/>
+      <c r="E26" s="48" t="n"/>
+      <c r="F26" s="48" t="n"/>
+      <c r="G26" s="48" t="n"/>
+      <c r="H26" s="48" t="n"/>
+      <c r="I26" s="48" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>Disc capacitor</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>0.1 µF 50 V ceramic, 2.5 mm pitch (C2, C6)</t>
+        </is>
+      </c>
+      <c r="C27" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E27" s="52">
+        <f>C27*D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G27" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H27" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I27" s="49" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>Bypass capacitor</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>0.1 µF 0805 (C3)</t>
+        </is>
+      </c>
+      <c r="C28" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E28" s="52">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G28" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H28" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I28" s="49" t="inlineStr">
+        <is>
+          <t>At the mux chip</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>1-Wire pull-up</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>4.7k ¼ W (R1)</t>
+        </is>
+      </c>
+      <c r="C29" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E29" s="52">
+        <f>C29*D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G29" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H29" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I29" s="49" t="inlineStr">
+        <is>
+          <t>DS18B20 bus</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>Opto series resistor</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>4.7k ½ W (R2, R4, R6, R8)</t>
+        </is>
+      </c>
+      <c r="C30" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E30" s="52">
+        <f>C30*D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G30" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H30" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I30" s="49" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>Opto pull-up resistor</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>10k ¼ W (R3, R5, R7, R9)</t>
+        </is>
+      </c>
+      <c r="C31" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E31" s="52">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G31" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H31" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I31" s="49" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>Mux pull-ups + reset</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>10k 0805 (R10–R20)</t>
+        </is>
+      </c>
+      <c r="C32" s="50" t="n">
+        <v>11</v>
+      </c>
+      <c r="D32" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E32" s="52">
+        <f>C32*D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G32" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H32" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I32" s="49" t="inlineStr">
+        <is>
+          <t>SDA/SCL pull-ups for each sensor channel, RESET pull-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="B33" s="48" t="n"/>
+      <c r="C33" s="48" t="n"/>
+      <c r="D33" s="48" t="n"/>
+      <c r="E33" s="48" t="n"/>
+      <c r="F33" s="48" t="n"/>
+      <c r="G33" s="48" t="n"/>
+      <c r="H33" s="48" t="n"/>
+      <c r="I33" s="48" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>Terminal header, 2-pos</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/2-G-5,08 (J1)</t>
+        </is>
+      </c>
+      <c r="C34" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="51" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E34" s="52">
+        <f>C34*D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G34" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H34" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I34" s="49" t="inlineStr">
+        <is>
+          <t>24 VAC in</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>Terminal plug, 2-pos</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/2-ST-5,08</t>
+        </is>
+      </c>
+      <c r="C35" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="51" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E35" s="52">
+        <f>C35*D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G35" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H35" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I35" s="49" t="inlineStr">
+        <is>
+          <t>Mates J1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>Terminal header, 4-pos</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/4-G-5,08 (J2, J5)</t>
+        </is>
+      </c>
+      <c r="C36" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="52">
+        <f>C36*D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G36" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H36" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I36" s="49" t="inlineStr">
+        <is>
+          <t>Thermostat calls; main I²C bus</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>Terminal plug, 4-pos</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Phoenix MC 1,5/4-ST-5,08</t>
+        </is>
+      </c>
+      <c r="C37" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="51" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E37" s="52">
+        <f>C37*D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G37" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H37" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I37" s="49" t="inlineStr">
+        <is>
+          <t>Mates J2, J5</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH header, 3-pin</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>B3B-XH-A (J3, J4)</t>
+        </is>
+      </c>
+      <c r="C38" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E38" s="52">
+        <f>C38*D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G38" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H38" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I38" s="49" t="inlineStr">
+        <is>
+          <t>DS18B20 probes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH header, 4-pin</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>B4B-XH-A (J6–J10)</t>
+        </is>
+      </c>
+      <c r="C39" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="D39" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E39" s="52">
+        <f>C39*D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G39" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H39" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I39" s="49" t="inlineStr">
+        <is>
+          <t>SHT45 ×2, SDP810 ×3 (mux channels 0–4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH housing, 3-pin</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>XHP-3 + SXH-001T-P0.6 crimps</t>
+        </is>
+      </c>
+      <c r="C40" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="51" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E40" s="52">
+        <f>C40*D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G40" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H40" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I40" s="49" t="inlineStr">
+        <is>
+          <t>Cable side</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>JST-XH housing, 4-pin</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>XHP-4 + SXH-001T-P0.6 crimps</t>
+        </is>
+      </c>
+      <c r="C41" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E41" s="52">
+        <f>C41*D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="39" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G41" s="54" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="H41" s="55" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="I41" s="49" t="inlineStr">
+        <is>
+          <t>Cable side</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="D43" s="42" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E43" s="43">
+        <f>SUM(E5:E41)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId32"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
@@ -5295,7 +8900,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6108,7 +9713,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>